<commit_message>
fix(tests): implement test and correct tests
</commit_message>
<xml_diff>
--- a/tests/data/example.xlsx
+++ b/tests/data/example.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="8"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Words" sheetId="1" state="visible" r:id="rId3"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="96">
   <si>
     <t xml:space="preserve">form</t>
   </si>
@@ -279,28 +279,25 @@
     <t xml:space="preserve">Wiktionnaire, Fondation Wikimédia</t>
   </si>
   <si>
-    <t xml:space="preserve">parl-+1sg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parle</t>
+    <t xml:space="preserve">manger+1sg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mange</t>
   </si>
   <si>
     <t xml:space="preserve">normal conjugation</t>
   </si>
   <si>
-    <t xml:space="preserve">dé-parl+inf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">déparler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dé-gagn+inf</t>
+    <t xml:space="preserve">dé-manger+inf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">démanger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dé-gagner+inf</t>
   </si>
   <si>
     <t xml:space="preserve">gagner does not select for dé-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parl</t>
   </si>
   <si>
     <t xml:space="preserve">bare stem not allowed</t>
@@ -1158,6 +1155,9 @@
   </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.44"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
@@ -1202,10 +1202,10 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="0" t="s">
         <v>90</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1229,10 +1229,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="0" t="s">
         <v>92</v>
-      </c>
-      <c r="B1" s="0" t="s">
-        <v>93</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>3</v>
@@ -1251,10 +1251,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1262,7 +1262,7 @@
         <v>76</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>